<commit_message>
Version 1.6: Change data source input.
</commit_message>
<xml_diff>
--- a/Downloaded/KDEHeader.xlsx
+++ b/Downloaded/KDEHeader.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="KDEHeader" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1564" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1969" uniqueCount="750">
   <si>
     <t>KDE00001</t>
   </si>
@@ -1823,13 +1824,460 @@
   </si>
   <si>
     <t>DataDomain</t>
+  </si>
+  <si>
+    <t>ElementName</t>
+  </si>
+  <si>
+    <t>PersonName</t>
+  </si>
+  <si>
+    <t>CommissionAmount</t>
+  </si>
+  <si>
+    <t>DistrictOverridingAmount</t>
+  </si>
+  <si>
+    <t>DistrictSpinOffAmount</t>
+  </si>
+  <si>
+    <t>DistrictTargetAmount</t>
+  </si>
+  <si>
+    <t>DivisionSpinOffAmount</t>
+  </si>
+  <si>
+    <t>RenewalYearCommission</t>
+  </si>
+  <si>
+    <t>RenewalYearCommissionAmount</t>
+  </si>
+  <si>
+    <t>StampDutyAmount</t>
+  </si>
+  <si>
+    <t>UnitOverridingAmount</t>
+  </si>
+  <si>
+    <t>UnitSpinOffAmount</t>
+  </si>
+  <si>
+    <t>BenefitPaymentDate</t>
+  </si>
+  <si>
+    <t>BenefitPaymentPeriod</t>
+  </si>
+  <si>
+    <t>BenefitPercentage</t>
+  </si>
+  <si>
+    <t>DividendAmount</t>
+  </si>
+  <si>
+    <t>DividendInterestAmount</t>
+  </si>
+  <si>
+    <t>BranchCode</t>
+  </si>
+  <si>
+    <t>BranchName</t>
+  </si>
+  <si>
+    <t>AccidentOccurredDate</t>
+  </si>
+  <si>
+    <t>AdmissionDate</t>
+  </si>
+  <si>
+    <t>ClaimIssueTypeCode</t>
+  </si>
+  <si>
+    <t>ClaimNumber</t>
+  </si>
+  <si>
+    <t>ClaimPaidAmount</t>
+  </si>
+  <si>
+    <t>ClaimPaymentDate</t>
+  </si>
+  <si>
+    <t>ClaimReceivedDate</t>
+  </si>
+  <si>
+    <t>ClaimReceivedNumber</t>
+  </si>
+  <si>
+    <t>ClaimRejectReason</t>
+  </si>
+  <si>
+    <t>ClaimStatusCode</t>
+  </si>
+  <si>
+    <t>ClaimSubmitChannelCode</t>
+  </si>
+  <si>
+    <t>ClaimTypeCode</t>
+  </si>
+  <si>
+    <t>IncurredAmount</t>
+  </si>
+  <si>
+    <t>MedicalConditionTypeCode</t>
+  </si>
+  <si>
+    <t>RiskCessationTerm</t>
+  </si>
+  <si>
+    <t>CoveragePlanCode</t>
+  </si>
+  <si>
+    <t>CoveragePlanName</t>
+  </si>
+  <si>
+    <t>CustomerIDNumber</t>
+  </si>
+  <si>
+    <t>EmployeeIDNumber</t>
+  </si>
+  <si>
+    <t>EndorsementNumber</t>
+  </si>
+  <si>
+    <t>FundIDNumber</t>
+  </si>
+  <si>
+    <t>FundOrderNumber</t>
+  </si>
+  <si>
+    <t>FundOrderTypeCode</t>
+  </si>
+  <si>
+    <t>BusinessGroupCode</t>
+  </si>
+  <si>
+    <t>BusinessTypeCode</t>
+  </si>
+  <si>
+    <t>GroupMemberTypeCode</t>
+  </si>
+  <si>
+    <t>GroupPlanCode</t>
+  </si>
+  <si>
+    <t>InsuredAttainedAge</t>
+  </si>
+  <si>
+    <t>RiskClassCode</t>
+  </si>
+  <si>
+    <t>LoanInterestAmount</t>
+  </si>
+  <si>
+    <t>PolicyDeliveryConfirmationDate</t>
+  </si>
+  <si>
+    <t>PolicyDispatchDate</t>
+  </si>
+  <si>
+    <t>MaturityDate</t>
+  </si>
+  <si>
+    <t>LoanApprovalDate</t>
+  </si>
+  <si>
+    <t>PolicyCertificationNumber</t>
+  </si>
+  <si>
+    <t>BankAccountNumber</t>
+  </si>
+  <si>
+    <t>BankBranchCode</t>
+  </si>
+  <si>
+    <t>BankCode</t>
+  </si>
+  <si>
+    <t>CreditCardNumber</t>
+  </si>
+  <si>
+    <t>PaymentMethodCode</t>
+  </si>
+  <si>
+    <t>PremiumPaymentSubmissionNumber</t>
+  </si>
+  <si>
+    <t>CommunicationContactMethodCode</t>
+  </si>
+  <si>
+    <t>CurrentAddress</t>
+  </si>
+  <si>
+    <t>EmailAddress</t>
+  </si>
+  <si>
+    <t>FATCAAnswer</t>
+  </si>
+  <si>
+    <t>FATCAStatus</t>
+  </si>
+  <si>
+    <t>HighestEducationLevelCode</t>
+  </si>
+  <si>
+    <t>HomePhoneNumber</t>
+  </si>
+  <si>
+    <t>HouseRegistrationAddress</t>
+  </si>
+  <si>
+    <t>IDTypeCode</t>
+  </si>
+  <si>
+    <t>MaritalStatusCode</t>
+  </si>
+  <si>
+    <t>MobilePhoneNumber</t>
+  </si>
+  <si>
+    <t>NationalityCode</t>
+  </si>
+  <si>
+    <t>OccupationClassCode</t>
+  </si>
+  <si>
+    <t>OccupationTypeCode</t>
+  </si>
+  <si>
+    <t>PassportNumber</t>
+  </si>
+  <si>
+    <t>PersonBirthDate</t>
+  </si>
+  <si>
+    <t>PersonDeadDate</t>
+  </si>
+  <si>
+    <t>PersonEnglishName</t>
+  </si>
+  <si>
+    <t>PersonGenderCode</t>
+  </si>
+  <si>
+    <t>PersonHeight</t>
+  </si>
+  <si>
+    <t>PersonRelationshipCode</t>
+  </si>
+  <si>
+    <t>PersonTitle</t>
+  </si>
+  <si>
+    <t>PersonTypeCode</t>
+  </si>
+  <si>
+    <t>PersonWeight</t>
+  </si>
+  <si>
+    <t>PesonTitle</t>
+  </si>
+  <si>
+    <t>TaxPayerIDNumber</t>
+  </si>
+  <si>
+    <t>TaxReductionConsentFlag</t>
+  </si>
+  <si>
+    <t>ThaiIDNumber</t>
+  </si>
+  <si>
+    <t>WorkPhoneNumber</t>
+  </si>
+  <si>
+    <t>WorkplaceAddress</t>
+  </si>
+  <si>
+    <t>WorkplacePhoneNumber</t>
+  </si>
+  <si>
+    <t>PolicyEffectiveDate</t>
+  </si>
+  <si>
+    <t>PolicyHolderAuthorityDelegationFlags</t>
+  </si>
+  <si>
+    <t>PolicyIssuanceDate</t>
+  </si>
+  <si>
+    <t>PolicyNumber</t>
+  </si>
+  <si>
+    <t>PolicyStatusCode</t>
+  </si>
+  <si>
+    <t>PolicyStatusDate</t>
+  </si>
+  <si>
+    <t>SumAssured</t>
+  </si>
+  <si>
+    <t>RiderEffectiveDate</t>
+  </si>
+  <si>
+    <t>RiderStatusCode</t>
+  </si>
+  <si>
+    <t>RiderStatusDate</t>
+  </si>
+  <si>
+    <t>InvoiceNumber</t>
+  </si>
+  <si>
+    <t>PaymentFrequency</t>
+  </si>
+  <si>
+    <t>PaymentFrequencyCode</t>
+  </si>
+  <si>
+    <t>PremiumAmount</t>
+  </si>
+  <si>
+    <t>PremiumCessationTerm</t>
+  </si>
+  <si>
+    <t>PremiumDueDate</t>
+  </si>
+  <si>
+    <t>PremiumPaymentPeriod</t>
+  </si>
+  <si>
+    <t>PremiumPaymentDate</t>
+  </si>
+  <si>
+    <t>PremiumReceiptIssueDate</t>
+  </si>
+  <si>
+    <t>PremiumReceiptNumber</t>
+  </si>
+  <si>
+    <t>ExperienceRefundRate</t>
+  </si>
+  <si>
+    <t>PremiumRefundDate</t>
+  </si>
+  <si>
+    <t>RefundCompleteDate</t>
+  </si>
+  <si>
+    <t>AdditionalRiderAllowedFlag</t>
+  </si>
+  <si>
+    <t>BasePlanCode</t>
+  </si>
+  <si>
+    <t>EntryAgeRange</t>
+  </si>
+  <si>
+    <t>MaximumCoverageTerm</t>
+  </si>
+  <si>
+    <t>MedicalCheckRequiredFlag</t>
+  </si>
+  <si>
+    <t>RiderName</t>
+  </si>
+  <si>
+    <t>RiderPlanCode</t>
+  </si>
+  <si>
+    <t>RiderSumAssuredAccumulatedFlag</t>
+  </si>
+  <si>
+    <t>SaleStartDate</t>
+  </si>
+  <si>
+    <t>ApplicationNumber</t>
+  </si>
+  <si>
+    <t>ApplicationStatusCode</t>
+  </si>
+  <si>
+    <t>ProposalDate</t>
+  </si>
+  <si>
+    <t>AgentHireStartDate</t>
+  </si>
+  <si>
+    <t>AgentIDNumber</t>
+  </si>
+  <si>
+    <t>AgentIncomeAmount</t>
+  </si>
+  <si>
+    <t>AgentLicenseExpiryDate</t>
+  </si>
+  <si>
+    <t>AgentLicenseNumber</t>
+  </si>
+  <si>
+    <t>AgentMeasureEndDate</t>
+  </si>
+  <si>
+    <t>AgentMeasureStartDate</t>
+  </si>
+  <si>
+    <t>AgentPosition</t>
+  </si>
+  <si>
+    <t>AgentQualificationTypeCode</t>
+  </si>
+  <si>
+    <t>AgentStructureID</t>
+  </si>
+  <si>
+    <t>BrokerName</t>
+  </si>
+  <si>
+    <t>FirstYearPremiumTarget</t>
+  </si>
+  <si>
+    <t>ParentStructureID</t>
+  </si>
+  <si>
+    <t>PercentageOfNewUnitsPerDistricts</t>
+  </si>
+  <si>
+    <t>SellingBranchCode</t>
+  </si>
+  <si>
+    <t>TrainingCourseStartDate</t>
+  </si>
+  <si>
+    <t>SurrenderChargeAmount</t>
+  </si>
+  <si>
+    <t>FreelookStatusCode</t>
+  </si>
+  <si>
+    <t>HealthCheckFlag</t>
+  </si>
+  <si>
+    <t>HealthCheckItemCode</t>
+  </si>
+  <si>
+    <t>HealthImpairmentFlag</t>
+  </si>
+  <si>
+    <t>HealthImpairmentNumber</t>
+  </si>
+  <si>
+    <t>Dup</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1865,6 +2313,14 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1898,13 +2354,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7816,4 +8273,2446 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E202"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="C1" t="s">
+        <v>749</v>
+      </c>
+      <c r="E1" s="6"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>671</v>
+      </c>
+      <c r="C2" t="b">
+        <f>A2=A1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>689</v>
+      </c>
+      <c r="C3" t="b">
+        <f>A3=A2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>691</v>
+      </c>
+      <c r="C4" t="b">
+        <f t="shared" ref="C4:C67" si="0">A4=A3</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>667</v>
+      </c>
+      <c r="C5" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>679</v>
+      </c>
+      <c r="C6" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" t="s">
+        <v>688</v>
+      </c>
+      <c r="C7" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>688</v>
+      </c>
+      <c r="C8" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>688</v>
+      </c>
+      <c r="C9" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>686</v>
+      </c>
+      <c r="C10" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>675</v>
+      </c>
+      <c r="C11" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>669</v>
+      </c>
+      <c r="C12" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" t="s">
+        <v>671</v>
+      </c>
+      <c r="C13" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>681</v>
+      </c>
+      <c r="C14" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" t="s">
+        <v>682</v>
+      </c>
+      <c r="C15" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" t="s">
+        <v>602</v>
+      </c>
+      <c r="C16" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
+        <v>602</v>
+      </c>
+      <c r="C17" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
+        <v>602</v>
+      </c>
+      <c r="C18" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" t="s">
+        <v>678</v>
+      </c>
+      <c r="C19" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" t="s">
+        <v>668</v>
+      </c>
+      <c r="C20" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" t="s">
+        <v>690</v>
+      </c>
+      <c r="C21" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" t="s">
+        <v>662</v>
+      </c>
+      <c r="C22" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>60</v>
+      </c>
+      <c r="B23" t="s">
+        <v>746</v>
+      </c>
+      <c r="C23" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" t="s">
+        <v>743</v>
+      </c>
+      <c r="C24" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" t="s">
+        <v>707</v>
+      </c>
+      <c r="C25" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" t="s">
+        <v>614</v>
+      </c>
+      <c r="C26" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" t="s">
+        <v>713</v>
+      </c>
+      <c r="C27" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>75</v>
+      </c>
+      <c r="B28" t="s">
+        <v>645</v>
+      </c>
+      <c r="C28" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" t="s">
+        <v>660</v>
+      </c>
+      <c r="C29" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30" t="s">
+        <v>673</v>
+      </c>
+      <c r="C30" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>84</v>
+      </c>
+      <c r="B31" t="s">
+        <v>674</v>
+      </c>
+      <c r="C31" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" t="s">
+        <v>644</v>
+      </c>
+      <c r="C32" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>90</v>
+      </c>
+      <c r="B33" t="s">
+        <v>643</v>
+      </c>
+      <c r="C33" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>93</v>
+      </c>
+      <c r="B34" t="s">
+        <v>676</v>
+      </c>
+      <c r="C34" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" t="s">
+        <v>647</v>
+      </c>
+      <c r="C35" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>99</v>
+      </c>
+      <c r="B36" t="s">
+        <v>637</v>
+      </c>
+      <c r="C36" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>102</v>
+      </c>
+      <c r="B37" t="s">
+        <v>670</v>
+      </c>
+      <c r="C37" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" t="s">
+        <v>672</v>
+      </c>
+      <c r="C38" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" t="s">
+        <v>663</v>
+      </c>
+      <c r="C39" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>111</v>
+      </c>
+      <c r="B40" t="s">
+        <v>623</v>
+      </c>
+      <c r="C40" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>114</v>
+      </c>
+      <c r="B41" t="s">
+        <v>623</v>
+      </c>
+      <c r="C41" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>117</v>
+      </c>
+      <c r="B42" t="s">
+        <v>661</v>
+      </c>
+      <c r="C42" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>120</v>
+      </c>
+      <c r="B43" t="s">
+        <v>628</v>
+      </c>
+      <c r="C43" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>123</v>
+      </c>
+      <c r="B44" t="s">
+        <v>633</v>
+      </c>
+      <c r="C44" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>126</v>
+      </c>
+      <c r="B45" t="s">
+        <v>630</v>
+      </c>
+      <c r="C45" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>129</v>
+      </c>
+      <c r="B46" t="s">
+        <v>631</v>
+      </c>
+      <c r="C46" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>132</v>
+      </c>
+      <c r="B47" t="s">
+        <v>632</v>
+      </c>
+      <c r="C47" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>135</v>
+      </c>
+      <c r="B48" t="s">
+        <v>624</v>
+      </c>
+      <c r="C48" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>138</v>
+      </c>
+      <c r="B49" t="s">
+        <v>659</v>
+      </c>
+      <c r="C49" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>141</v>
+      </c>
+      <c r="B50" t="s">
+        <v>712</v>
+      </c>
+      <c r="C50" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>144</v>
+      </c>
+      <c r="B51" t="s">
+        <v>620</v>
+      </c>
+      <c r="C51" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>144</v>
+      </c>
+      <c r="B52" t="s">
+        <v>621</v>
+      </c>
+      <c r="C52" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>144</v>
+      </c>
+      <c r="B53" t="s">
+        <v>677</v>
+      </c>
+      <c r="C53" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>147</v>
+      </c>
+      <c r="B54" t="s">
+        <v>621</v>
+      </c>
+      <c r="C54" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>150</v>
+      </c>
+      <c r="B55" t="s">
+        <v>625</v>
+      </c>
+      <c r="C55" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>156</v>
+      </c>
+      <c r="B56" t="s">
+        <v>626</v>
+      </c>
+      <c r="C56" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>159</v>
+      </c>
+      <c r="B57" t="s">
+        <v>627</v>
+      </c>
+      <c r="C57" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>162</v>
+      </c>
+      <c r="B58" t="s">
+        <v>622</v>
+      </c>
+      <c r="C58" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>165</v>
+      </c>
+      <c r="B59" t="s">
+        <v>631</v>
+      </c>
+      <c r="C59" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>168</v>
+      </c>
+      <c r="B60" t="s">
+        <v>671</v>
+      </c>
+      <c r="C60" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>171</v>
+      </c>
+      <c r="B61" t="s">
+        <v>671</v>
+      </c>
+      <c r="C61" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>174</v>
+      </c>
+      <c r="B62" t="s">
+        <v>731</v>
+      </c>
+      <c r="C62" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>177</v>
+      </c>
+      <c r="B63" t="s">
+        <v>728</v>
+      </c>
+      <c r="C63" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>180</v>
+      </c>
+      <c r="B64" t="s">
+        <v>602</v>
+      </c>
+      <c r="C64" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>183</v>
+      </c>
+      <c r="B65" t="s">
+        <v>728</v>
+      </c>
+      <c r="C65" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>186</v>
+      </c>
+      <c r="B66" t="s">
+        <v>638</v>
+      </c>
+      <c r="C66" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>189</v>
+      </c>
+      <c r="B67" t="s">
+        <v>655</v>
+      </c>
+      <c r="C67" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>192</v>
+      </c>
+      <c r="B68" t="s">
+        <v>730</v>
+      </c>
+      <c r="C68" t="b">
+        <f t="shared" ref="C68:C131" si="1">A68=A67</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>195</v>
+      </c>
+      <c r="B69" t="s">
+        <v>656</v>
+      </c>
+      <c r="C69" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>198</v>
+      </c>
+      <c r="B70" t="s">
+        <v>692</v>
+      </c>
+      <c r="C70" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>201</v>
+      </c>
+      <c r="B71" t="s">
+        <v>719</v>
+      </c>
+      <c r="C71" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>201</v>
+      </c>
+      <c r="B72" t="s">
+        <v>745</v>
+      </c>
+      <c r="C72" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>204</v>
+      </c>
+      <c r="B73" t="s">
+        <v>741</v>
+      </c>
+      <c r="C73" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>207</v>
+      </c>
+      <c r="B74" t="s">
+        <v>618</v>
+      </c>
+      <c r="C74" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>207</v>
+      </c>
+      <c r="B75" t="s">
+        <v>619</v>
+      </c>
+      <c r="C75" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>210</v>
+      </c>
+      <c r="B76" t="s">
+        <v>618</v>
+      </c>
+      <c r="C76" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>213</v>
+      </c>
+      <c r="B77" t="s">
+        <v>616</v>
+      </c>
+      <c r="C77" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>216</v>
+      </c>
+      <c r="B78" t="s">
+        <v>705</v>
+      </c>
+      <c r="C78" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>219</v>
+      </c>
+      <c r="B79" t="s">
+        <v>705</v>
+      </c>
+      <c r="C79" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>222</v>
+      </c>
+      <c r="B80" t="s">
+        <v>705</v>
+      </c>
+      <c r="C80" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>225</v>
+      </c>
+      <c r="B81" t="s">
+        <v>705</v>
+      </c>
+      <c r="C81" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>228</v>
+      </c>
+      <c r="B82" t="s">
+        <v>705</v>
+      </c>
+      <c r="C82" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>231</v>
+      </c>
+      <c r="B83" t="s">
+        <v>705</v>
+      </c>
+      <c r="C83" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>234</v>
+      </c>
+      <c r="B84" t="s">
+        <v>703</v>
+      </c>
+      <c r="C84" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>234</v>
+      </c>
+      <c r="B85" t="s">
+        <v>704</v>
+      </c>
+      <c r="C85" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>237</v>
+      </c>
+      <c r="B86" t="s">
+        <v>708</v>
+      </c>
+      <c r="C86" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>240</v>
+      </c>
+      <c r="B87" t="s">
+        <v>708</v>
+      </c>
+      <c r="C87" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>243</v>
+      </c>
+      <c r="B88" t="s">
+        <v>705</v>
+      </c>
+      <c r="C88" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>246</v>
+      </c>
+      <c r="B89" t="s">
+        <v>705</v>
+      </c>
+      <c r="C89" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>249</v>
+      </c>
+      <c r="B90" t="s">
+        <v>695</v>
+      </c>
+      <c r="C90" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>252</v>
+      </c>
+      <c r="B91" t="s">
+        <v>695</v>
+      </c>
+      <c r="C91" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>255</v>
+      </c>
+      <c r="B92" t="s">
+        <v>724</v>
+      </c>
+      <c r="C92" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>258</v>
+      </c>
+      <c r="B93" t="s">
+        <v>724</v>
+      </c>
+      <c r="C93" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>261</v>
+      </c>
+      <c r="B94" t="s">
+        <v>711</v>
+      </c>
+      <c r="C94" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>264</v>
+      </c>
+      <c r="B95" t="s">
+        <v>711</v>
+      </c>
+      <c r="C95" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>267</v>
+      </c>
+      <c r="B96" t="s">
+        <v>710</v>
+      </c>
+      <c r="C96" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>270</v>
+      </c>
+      <c r="B97" t="s">
+        <v>748</v>
+      </c>
+      <c r="C97" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>273</v>
+      </c>
+      <c r="B98" t="s">
+        <v>654</v>
+      </c>
+      <c r="C98" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>276</v>
+      </c>
+      <c r="B99" t="s">
+        <v>648</v>
+      </c>
+      <c r="C99" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>279</v>
+      </c>
+      <c r="B100" t="s">
+        <v>646</v>
+      </c>
+      <c r="C100" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>282</v>
+      </c>
+      <c r="B101" t="s">
+        <v>635</v>
+      </c>
+      <c r="C101" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>282</v>
+      </c>
+      <c r="B102" t="s">
+        <v>716</v>
+      </c>
+      <c r="C102" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>285</v>
+      </c>
+      <c r="B103" t="s">
+        <v>636</v>
+      </c>
+      <c r="C103" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>285</v>
+      </c>
+      <c r="B104" t="s">
+        <v>720</v>
+      </c>
+      <c r="C104" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>288</v>
+      </c>
+      <c r="B105" t="s">
+        <v>635</v>
+      </c>
+      <c r="C105" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>288</v>
+      </c>
+      <c r="B106" t="s">
+        <v>721</v>
+      </c>
+      <c r="C106" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>291</v>
+      </c>
+      <c r="B107" t="s">
+        <v>702</v>
+      </c>
+      <c r="C107" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>294</v>
+      </c>
+      <c r="B108" t="s">
+        <v>698</v>
+      </c>
+      <c r="C108" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>297</v>
+      </c>
+      <c r="B109" t="s">
+        <v>698</v>
+      </c>
+      <c r="C109" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>300</v>
+      </c>
+      <c r="B110" t="s">
+        <v>698</v>
+      </c>
+      <c r="C110" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>303</v>
+      </c>
+      <c r="B111" t="s">
+        <v>709</v>
+      </c>
+      <c r="C111" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>303</v>
+      </c>
+      <c r="B112" t="s">
+        <v>710</v>
+      </c>
+      <c r="C112" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>306</v>
+      </c>
+      <c r="B113" t="s">
+        <v>709</v>
+      </c>
+      <c r="C113" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>309</v>
+      </c>
+      <c r="B114" t="s">
+        <v>706</v>
+      </c>
+      <c r="C114" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>312</v>
+      </c>
+      <c r="B115" t="s">
+        <v>634</v>
+      </c>
+      <c r="C115" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>312</v>
+      </c>
+      <c r="B116" t="s">
+        <v>706</v>
+      </c>
+      <c r="C116" t="b">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>315</v>
+      </c>
+      <c r="B117" t="s">
+        <v>640</v>
+      </c>
+      <c r="C117" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>318</v>
+      </c>
+      <c r="B118" t="s">
+        <v>697</v>
+      </c>
+      <c r="C118" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>321</v>
+      </c>
+      <c r="B119" t="s">
+        <v>653</v>
+      </c>
+      <c r="C119" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>324</v>
+      </c>
+      <c r="B120" t="s">
+        <v>617</v>
+      </c>
+      <c r="C120" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>327</v>
+      </c>
+      <c r="B121" t="s">
+        <v>649</v>
+      </c>
+      <c r="C121" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>330</v>
+      </c>
+      <c r="B122" t="s">
+        <v>651</v>
+      </c>
+      <c r="C122" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>333</v>
+      </c>
+      <c r="B123" t="s">
+        <v>659</v>
+      </c>
+      <c r="C123" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>336</v>
+      </c>
+      <c r="B124" t="s">
+        <v>659</v>
+      </c>
+      <c r="C124" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>339</v>
+      </c>
+      <c r="B125" t="s">
+        <v>700</v>
+      </c>
+      <c r="C125" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>342</v>
+      </c>
+      <c r="B126" t="s">
+        <v>714</v>
+      </c>
+      <c r="C126" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>345</v>
+      </c>
+      <c r="B127" t="s">
+        <v>652</v>
+      </c>
+      <c r="C127" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>348</v>
+      </c>
+      <c r="B128" t="s">
+        <v>613</v>
+      </c>
+      <c r="C128" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>351</v>
+      </c>
+      <c r="B129" t="s">
+        <v>726</v>
+      </c>
+      <c r="C129" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>354</v>
+      </c>
+      <c r="B130" t="s">
+        <v>694</v>
+      </c>
+      <c r="C130" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>357</v>
+      </c>
+      <c r="B131" t="s">
+        <v>610</v>
+      </c>
+      <c r="C131" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>360</v>
+      </c>
+      <c r="B132" t="s">
+        <v>615</v>
+      </c>
+      <c r="C132" t="b">
+        <f t="shared" ref="C132:C195" si="2">A132=A131</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>363</v>
+      </c>
+      <c r="B133" t="s">
+        <v>680</v>
+      </c>
+      <c r="C133" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>366</v>
+      </c>
+      <c r="B134" t="s">
+        <v>684</v>
+      </c>
+      <c r="C134" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>369</v>
+      </c>
+      <c r="B135" t="s">
+        <v>687</v>
+      </c>
+      <c r="C135" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>372</v>
+      </c>
+      <c r="B136" t="s">
+        <v>665</v>
+      </c>
+      <c r="C136" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>375</v>
+      </c>
+      <c r="B137" t="s">
+        <v>664</v>
+      </c>
+      <c r="C137" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>378</v>
+      </c>
+      <c r="B138" t="s">
+        <v>658</v>
+      </c>
+      <c r="C138" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>381</v>
+      </c>
+      <c r="B139" t="s">
+        <v>657</v>
+      </c>
+      <c r="C139" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>384</v>
+      </c>
+      <c r="B140" t="s">
+        <v>629</v>
+      </c>
+      <c r="C140" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>387</v>
+      </c>
+      <c r="B141" t="s">
+        <v>747</v>
+      </c>
+      <c r="C141" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>390</v>
+      </c>
+      <c r="B142" t="s">
+        <v>737</v>
+      </c>
+      <c r="C142" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>393</v>
+      </c>
+      <c r="B143" t="s">
+        <v>696</v>
+      </c>
+      <c r="C143" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>396</v>
+      </c>
+      <c r="B144" t="s">
+        <v>663</v>
+      </c>
+      <c r="C144" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>399</v>
+      </c>
+      <c r="B145" t="s">
+        <v>744</v>
+      </c>
+      <c r="C145" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>402</v>
+      </c>
+      <c r="B146" t="s">
+        <v>641</v>
+      </c>
+      <c r="C146" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>405</v>
+      </c>
+      <c r="B147" t="s">
+        <v>642</v>
+      </c>
+      <c r="C147" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>408</v>
+      </c>
+      <c r="B148" t="s">
+        <v>639</v>
+      </c>
+      <c r="C148" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>411</v>
+      </c>
+      <c r="B149" t="s">
+        <v>725</v>
+      </c>
+      <c r="C149" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>414</v>
+      </c>
+      <c r="B150" t="s">
+        <v>693</v>
+      </c>
+      <c r="C150" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>417</v>
+      </c>
+      <c r="B151" t="s">
+        <v>734</v>
+      </c>
+      <c r="C151" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>420</v>
+      </c>
+      <c r="B152" t="s">
+        <v>736</v>
+      </c>
+      <c r="C152" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>423</v>
+      </c>
+      <c r="B153" t="s">
+        <v>739</v>
+      </c>
+      <c r="C153" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>426</v>
+      </c>
+      <c r="B154" t="s">
+        <v>738</v>
+      </c>
+      <c r="C154" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>429</v>
+      </c>
+      <c r="B155" t="s">
+        <v>679</v>
+      </c>
+      <c r="C155" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>435</v>
+      </c>
+      <c r="B156" t="s">
+        <v>666</v>
+      </c>
+      <c r="C156" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>438</v>
+      </c>
+      <c r="B157" t="s">
+        <v>670</v>
+      </c>
+      <c r="C157" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>441</v>
+      </c>
+      <c r="B158" t="s">
+        <v>603</v>
+      </c>
+      <c r="C158" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>444</v>
+      </c>
+      <c r="B159" t="s">
+        <v>608</v>
+      </c>
+      <c r="C159" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>444</v>
+      </c>
+      <c r="B160" t="s">
+        <v>609</v>
+      </c>
+      <c r="C160" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>447</v>
+      </c>
+      <c r="B161" t="s">
+        <v>604</v>
+      </c>
+      <c r="C161" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>450</v>
+      </c>
+      <c r="B162" t="s">
+        <v>611</v>
+      </c>
+      <c r="C162" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>453</v>
+      </c>
+      <c r="B163" t="s">
+        <v>605</v>
+      </c>
+      <c r="C163" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>456</v>
+      </c>
+      <c r="B164" t="s">
+        <v>607</v>
+      </c>
+      <c r="C164" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>459</v>
+      </c>
+      <c r="B165" t="s">
+        <v>612</v>
+      </c>
+      <c r="C165" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>462</v>
+      </c>
+      <c r="B166" t="s">
+        <v>606</v>
+      </c>
+      <c r="C166" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>465</v>
+      </c>
+      <c r="B167" t="s">
+        <v>711</v>
+      </c>
+      <c r="C167" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>468</v>
+      </c>
+      <c r="B168" t="s">
+        <v>729</v>
+      </c>
+      <c r="C168" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>471</v>
+      </c>
+      <c r="B169" t="s">
+        <v>742</v>
+      </c>
+      <c r="C169" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>474</v>
+      </c>
+      <c r="B170" t="s">
+        <v>727</v>
+      </c>
+      <c r="C170" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>477</v>
+      </c>
+      <c r="B171" t="s">
+        <v>735</v>
+      </c>
+      <c r="C171" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>480</v>
+      </c>
+      <c r="B172" t="s">
+        <v>671</v>
+      </c>
+      <c r="C172" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>483</v>
+      </c>
+      <c r="B173" t="s">
+        <v>676</v>
+      </c>
+      <c r="C173" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>486</v>
+      </c>
+      <c r="B174" t="s">
+        <v>655</v>
+      </c>
+      <c r="C174" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>491</v>
+      </c>
+      <c r="B175" t="s">
+        <v>740</v>
+      </c>
+      <c r="C175" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>494</v>
+      </c>
+      <c r="B176" t="s">
+        <v>682</v>
+      </c>
+      <c r="C176" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>497</v>
+      </c>
+      <c r="B177" t="s">
+        <v>655</v>
+      </c>
+      <c r="C177" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>500</v>
+      </c>
+      <c r="B178" t="s">
+        <v>671</v>
+      </c>
+      <c r="C178" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>503</v>
+      </c>
+      <c r="B179" t="s">
+        <v>679</v>
+      </c>
+      <c r="C179" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>506</v>
+      </c>
+      <c r="B180" t="s">
+        <v>685</v>
+      </c>
+      <c r="C180" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>509</v>
+      </c>
+      <c r="B181" t="s">
+        <v>602</v>
+      </c>
+      <c r="C181" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>512</v>
+      </c>
+      <c r="B182" t="s">
+        <v>663</v>
+      </c>
+      <c r="C182" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>518</v>
+      </c>
+      <c r="B183" t="s">
+        <v>676</v>
+      </c>
+      <c r="C183" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>521</v>
+      </c>
+      <c r="B184" t="s">
+        <v>602</v>
+      </c>
+      <c r="C184" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>524</v>
+      </c>
+      <c r="B185" t="s">
+        <v>682</v>
+      </c>
+      <c r="C185" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>527</v>
+      </c>
+      <c r="B186" t="s">
+        <v>602</v>
+      </c>
+      <c r="C186" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>530</v>
+      </c>
+      <c r="B187" t="s">
+        <v>602</v>
+      </c>
+      <c r="C187" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>533</v>
+      </c>
+      <c r="B188" t="s">
+        <v>683</v>
+      </c>
+      <c r="C188" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>536</v>
+      </c>
+      <c r="B189" t="s">
+        <v>676</v>
+      </c>
+      <c r="C189" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>539</v>
+      </c>
+      <c r="B190" t="s">
+        <v>688</v>
+      </c>
+      <c r="C190" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>542</v>
+      </c>
+      <c r="B191" t="s">
+        <v>705</v>
+      </c>
+      <c r="C191" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>545</v>
+      </c>
+      <c r="B192" t="s">
+        <v>701</v>
+      </c>
+      <c r="C192" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>548</v>
+      </c>
+      <c r="B193" t="s">
+        <v>699</v>
+      </c>
+      <c r="C193" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>551</v>
+      </c>
+      <c r="B194" t="s">
+        <v>723</v>
+      </c>
+      <c r="C194" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>554</v>
+      </c>
+      <c r="B195" t="s">
+        <v>717</v>
+      </c>
+      <c r="C195" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>557</v>
+      </c>
+      <c r="B196" t="s">
+        <v>715</v>
+      </c>
+      <c r="C196" t="b">
+        <f t="shared" ref="C196:C202" si="3">A196=A195</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>560</v>
+      </c>
+      <c r="B197" t="s">
+        <v>722</v>
+      </c>
+      <c r="C197" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>566</v>
+      </c>
+      <c r="B198" t="s">
+        <v>718</v>
+      </c>
+      <c r="C198" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>569</v>
+      </c>
+      <c r="B199" t="s">
+        <v>733</v>
+      </c>
+      <c r="C199" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>572</v>
+      </c>
+      <c r="B200" t="s">
+        <v>732</v>
+      </c>
+      <c r="C200" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>575</v>
+      </c>
+      <c r="B201" t="s">
+        <v>688</v>
+      </c>
+      <c r="C201" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>578</v>
+      </c>
+      <c r="B202" t="s">
+        <v>650</v>
+      </c>
+      <c r="C202" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState ref="A2:B202">
+    <sortCondition ref="A2:A202"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>